<commit_message>
feat: add V2.4 testcase XML snapshots
</commit_message>
<xml_diff>
--- a/testcase/payment2.xlsx
+++ b/testcase/payment2.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="43">
   <si>
     <t>This document was exported from Numbers. Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -78,6 +78,9 @@
     <t>標籤</t>
   </si>
   <si>
+    <t>案例描述</t>
+  </si>
+  <si>
     <t>扣賬帳號</t>
   </si>
   <si>
@@ -102,6 +105,10 @@
     <t>耗時毫秒</t>
   </si>
   <si>
+    <t>test
+multi lines</t>
+  </si>
+  <si>
     <t>CT001</t>
   </si>
   <si>
@@ -109,6 +116,11 @@
   </si>
   <si>
     <t>smoke,regression</t>
+  </si>
+  <si>
+    <t>abc測試流程：
+1. Precheck
+2. Confirm</t>
   </si>
   <si>
     <t>1000000000</t>
@@ -139,6 +151,9 @@
     </r>
   </si>
   <si>
+    <t>No use</t>
+  </si>
+  <si>
     <t>CT002</t>
   </si>
   <si>
@@ -146,6 +161,10 @@
   </si>
   <si>
     <t>edge,amount</t>
+  </si>
+  <si>
+    <t>“test” &gt; 
+multiple lines</t>
   </si>
   <si>
     <t>1000000001</t>
@@ -508,7 +527,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -614,17 +633,20 @@
     <xf numFmtId="49" fontId="0" fillId="6" borderId="17" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
@@ -1842,18 +1864,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="2" width="16" style="25" customWidth="1"/>
     <col min="3" max="3" width="24" style="25" customWidth="1"/>
     <col min="4" max="4" width="16" style="25" customWidth="1"/>
-    <col min="5" max="6" width="10.1719" style="25" customWidth="1"/>
-    <col min="7" max="7" width="6" style="25" customWidth="1"/>
-    <col min="8" max="8" width="4.5" style="25" customWidth="1"/>
-    <col min="9" max="9" width="23" style="25" customWidth="1"/>
-    <col min="10" max="13" width="8.17188" style="25" customWidth="1"/>
-    <col min="14" max="16384" width="8.85156" style="25" customWidth="1"/>
+    <col min="5" max="5" width="18.5625" style="25" customWidth="1"/>
+    <col min="6" max="7" width="10.1719" style="25" customWidth="1"/>
+    <col min="8" max="8" width="6" style="25" customWidth="1"/>
+    <col min="9" max="9" width="4.5" style="25" customWidth="1"/>
+    <col min="10" max="10" width="23" style="25" customWidth="1"/>
+    <col min="11" max="14" width="8.17188" style="25" customWidth="1"/>
+    <col min="15" max="16384" width="8.85156" style="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1868,12 +1891,13 @@
       <c r="G1" s="27"/>
       <c r="H1" s="27"/>
       <c r="I1" s="27"/>
-      <c r="J1" t="s" s="28">
+      <c r="J1" s="27"/>
+      <c r="K1" t="s" s="28">
         <v>11</v>
       </c>
-      <c r="K1" s="27"/>
       <c r="L1" s="27"/>
       <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" t="s" s="29">
@@ -1903,95 +1927,109 @@
       <c r="I2" t="s" s="30">
         <v>20</v>
       </c>
-      <c r="J2" t="s" s="31">
+      <c r="J2" t="s" s="30">
         <v>21</v>
       </c>
-      <c r="K2" t="s" s="32">
+      <c r="K2" t="s" s="31">
         <v>22</v>
       </c>
-      <c r="L2" t="s" s="33">
+      <c r="L2" t="s" s="32">
+        <v>23</v>
+      </c>
+      <c r="M2" t="s" s="33">
         <v>11</v>
       </c>
-      <c r="M2" t="s" s="34">
-        <v>23</v>
+      <c r="N2" t="s" s="34">
+        <v>24</v>
       </c>
     </row>
     <row r="3" ht="68" customHeight="1">
-      <c r="A3" s="35"/>
-      <c r="B3" t="s" s="36">
-        <v>24</v>
-      </c>
-      <c r="C3" t="s" s="36">
+      <c r="A3" t="s" s="36">
         <v>25</v>
       </c>
-      <c r="D3" t="s" s="36">
+      <c r="B3" t="s" s="37">
         <v>26</v>
       </c>
-      <c r="E3" t="s" s="36">
+      <c r="C3" t="s" s="37">
         <v>27</v>
       </c>
-      <c r="F3" t="s" s="36">
+      <c r="D3" t="s" s="37">
         <v>28</v>
       </c>
-      <c r="G3" s="37">
+      <c r="E3" t="s" s="38">
+        <v>29</v>
+      </c>
+      <c r="F3" t="s" s="37">
+        <v>30</v>
+      </c>
+      <c r="G3" t="s" s="37">
+        <v>31</v>
+      </c>
+      <c r="H3" s="39">
         <v>100</v>
       </c>
-      <c r="H3" t="s" s="36">
-        <v>29</v>
-      </c>
-      <c r="I3" t="s" s="38">
-        <v>30</v>
-      </c>
-      <c r="J3" s="39"/>
-      <c r="K3" s="39"/>
-      <c r="L3" s="39"/>
+      <c r="I3" t="s" s="37">
+        <v>32</v>
+      </c>
+      <c r="J3" t="s" s="38">
+        <v>33</v>
+      </c>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
       <c r="M3" s="40"/>
+      <c r="N3" s="41"/>
     </row>
     <row r="4" ht="68" customHeight="1">
-      <c r="A4" s="35"/>
-      <c r="B4" t="s" s="36">
-        <v>31</v>
-      </c>
-      <c r="C4" t="s" s="36">
-        <v>32</v>
-      </c>
-      <c r="D4" t="s" s="36">
-        <v>33</v>
-      </c>
-      <c r="E4" t="s" s="36">
+      <c r="A4" t="s" s="35">
         <v>34</v>
       </c>
-      <c r="F4" t="s" s="36">
+      <c r="B4" t="s" s="37">
         <v>35</v>
       </c>
-      <c r="G4" s="37">
+      <c r="C4" t="s" s="37">
+        <v>36</v>
+      </c>
+      <c r="D4" t="s" s="37">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s" s="38">
+        <v>38</v>
+      </c>
+      <c r="F4" t="s" s="37">
+        <v>39</v>
+      </c>
+      <c r="G4" t="s" s="37">
+        <v>40</v>
+      </c>
+      <c r="H4" s="39">
         <v>0.01</v>
       </c>
-      <c r="H4" t="s" s="36">
-        <v>36</v>
-      </c>
-      <c r="I4" t="s" s="38">
-        <v>37</v>
-      </c>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
+      <c r="I4" t="s" s="37">
+        <v>41</v>
+      </c>
+      <c r="J4" t="s" s="38">
+        <v>42</v>
+      </c>
+      <c r="K4" s="40"/>
+      <c r="L4" s="40"/>
       <c r="M4" s="40"/>
+      <c r="N4" s="41"/>
     </row>
     <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" s="41"/>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="42"/>
-      <c r="L5" s="42"/>
+      <c r="A5" s="42"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
+      <c r="I5" s="43"/>
+      <c r="J5" s="43"/>
+      <c r="K5" s="43"/>
+      <c r="L5" s="43"/>
       <c r="M5" s="43"/>
+      <c r="N5" s="44"/>
     </row>
     <row r="6" ht="13.55" customHeight="1">
       <c r="A6" s="10"/>
@@ -2006,7 +2044,8 @@
       <c r="J6" s="11"/>
       <c r="K6" s="11"/>
       <c r="L6" s="11"/>
-      <c r="M6" s="12"/>
+      <c r="M6" s="11"/>
+      <c r="N6" s="12"/>
     </row>
     <row r="7" ht="13.55" customHeight="1">
       <c r="A7" s="10"/>
@@ -2021,7 +2060,8 @@
       <c r="J7" s="11"/>
       <c r="K7" s="11"/>
       <c r="L7" s="11"/>
-      <c r="M7" s="12"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="12"/>
     </row>
     <row r="8" ht="13.55" customHeight="1">
       <c r="A8" s="10"/>
@@ -2036,7 +2076,8 @@
       <c r="J8" s="11"/>
       <c r="K8" s="11"/>
       <c r="L8" s="11"/>
-      <c r="M8" s="12"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="12"/>
     </row>
     <row r="9" ht="13.55" customHeight="1">
       <c r="A9" s="10"/>
@@ -2051,27 +2092,29 @@
       <c r="J9" s="11"/>
       <c r="K9" s="11"/>
       <c r="L9" s="11"/>
-      <c r="M9" s="12"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="12"/>
     </row>
     <row r="10" ht="13.55" customHeight="1">
       <c r="A10" s="20"/>
-      <c r="B10" s="44"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="44"/>
-      <c r="K10" s="44"/>
-      <c r="L10" s="44"/>
-      <c r="M10" s="24"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="45"/>
+      <c r="J10" s="45"/>
+      <c r="K10" s="45"/>
+      <c r="L10" s="45"/>
+      <c r="M10" s="45"/>
+      <c r="N10" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="K1:N1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>